<commit_message>
nii-frontier: simplify engine API - MAKE_CURVE takes one two-column fedMoves range, drop scale arg, rename SWAP_NET->SWAP; rebuild simple workbook (single FOMC block, cleaner formulas) and master VBA with plain-language guide; golden values reconfirmed
</commit_message>
<xml_diff>
--- a/projects/nii-frontier/tools/NII_Engine_Simple.xlsx
+++ b/projects/nii-frontier/tools/NII_Engine_Simple.xlsx
@@ -58,13 +58,13 @@
       <color rgb="000000FF"/>
     </font>
     <font>
-      <name val="Consolas"/>
-      <color rgb="007F4F00"/>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <color rgb="00595959"/>
+      <name val="Consolas"/>
+      <color rgb="007F4F00"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -107,21 +107,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -196,17 +195,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblHolidays" displayName="tblHolidays" ref="A4:B10" headerRowCount="1">
-  <autoFilter ref="A4:B10"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Date"/>
-    <tableColumn id="2" name="Name"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight15" showRowStripes="1"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -498,10 +486,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="92" customWidth="1" min="1" max="1"/>
+    <col width="88" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -517,97 +505,90 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Minimal workbook to test the engine: build a calendar and a curve, then</t>
+          <t>Four functions: FED_HOL, MAKE_CURVE, ACCRUE, SWAP.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>accrue interest and price a swap month. No formulas ship; you add the VBA,</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>then paste the formulas from column E of the MODEL sheet.</t>
+          <t>SETUP</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>1. Open NII_ENGINE_ALL_VBA.txt. Alt+F11 in Excel.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SETUP</t>
+          <t>2. Paste its 6 modules. cCalendar and cStripCurve are CLASS modules;</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>1. Open NII_ENGINE_ALL_VBA.txt (6 modules, banner-separated).</t>
+          <t xml:space="preserve">   the other four are normal modules. Delete each block's first</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2. Alt+F11. Per module: Insert &gt; Module (CLASS Module for cCalendar &amp;</t>
+          <t xml:space="preserve">   'Attribute VB_Name' line. Rename each module to its banner name.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   cStripCurve), rename, paste body, skip the 'Attribute VB_Name' line.</t>
+          <t>3. Save as .xlsm. Press Ctrl+Alt+F9.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>3. Save as .xlsm. Press Ctrl+Alt+F9.</t>
+          <t>4. Go to MODEL. Copy each formula in column E into the yellow cell on</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>4. MODEL: paste each column-E formula into the yellow cell on its left</t>
+          <t xml:space="preserve">   its left. Do B4 (calendar) and B5 (curve) FIRST.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (B4 calendar, B5 curve first).</t>
+          <t>5. Each Result should match the Expected value next to it.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>5. Results should match the Expected column.</t>
+          <t>6. Alt+F8 &gt; TestAll writes a TESTS sheet — expect MODEL STATUS: OK.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>6. Alt+F8 &gt; TestAll -&gt; TESTS sheet, expect MODEL STATUS: OK.</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>RULE: handles flow cell-to-cell (B4, B5) — never type the handle as text.</t>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>RULE: ACCRUE and SWAP point at the curve CELL B5 — never type "cuts".</t>
         </is>
       </c>
     </row>
@@ -622,163 +603,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>INPUTS — objects rebuild from here on recalc</t>
+          <t>INPUTS</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>HOLIDAYS (Excel Table — add rows freely)</t>
+          <t>Holidays</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>SCENARIO 'cuts' — FOMC moves</t>
+          <t>FOMC moves (date | bps)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Move bps</t>
-        </is>
+      <c r="A4" s="5" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>-25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>New Year</t>
-        </is>
+        <v>46041</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>46190</v>
-      </c>
-      <c r="E5" s="7" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E5" s="6" t="n">
         <v>-25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>46041</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>MLK Day</t>
-        </is>
+        <v>46206</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>46232</v>
-      </c>
-      <c r="E6" s="7" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>-25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>46206</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Independence (obs)</t>
-        </is>
+        <v>46272</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>46281</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>-25</v>
+        <v>46323</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>46272</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Labor Day</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>46323</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>0</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>46352</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Thanksgiving</t>
-        </is>
+        <v>46381</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>46381</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Christmas</t>
-        </is>
-      </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Initial SOFR (%)</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="n">
+          <t>SOFR now %</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
         <v>3.8</v>
       </c>
     </row>
-    <row r="11">
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Scale ×</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>1</v>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Holidays = A4:A9   ·   FOMC = D4:E7   ·   SOFR = E10</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -788,14 +712,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -808,244 +732,218 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>1 · OBJECTS</t>
+          <t>1 · BUILD OBJECTS (do these first)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>FORMULA TO PASTE</t>
+          <t>PASTE THIS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Calendar handle</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="B4" s="9" t="n"/>
       <c r="E4" s="10">
-        <f>FED_HOL(tblHolidays[Date])</f>
+        <f>FED_HOL(INPUTS!A4:A9)</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Curve handle</t>
+          <t>Curve</t>
         </is>
       </c>
       <c r="B5" s="9" t="n"/>
       <c r="E5" s="10">
-        <f>MAKE_CURVE("cuts",INPUTS!E10,INPUTS!D5:D8,INPUTS!E5:E8,INPUTS!E11,$B$4)</f>
+        <f>MAKE_CURVE("cuts",INPUTS!E10,INPUTS!D4:E7,$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2 · ACCRUALS</t>
+          <t>2 · ACCRUE</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Expected</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Expected</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>FORMULA TO PASTE</t>
+          <t>PASTE THIS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ON, normal (15-Jul)</t>
+          <t>ON, normal day</t>
         </is>
       </c>
       <c r="B8" s="11" t="n"/>
-      <c r="C8" s="4">
-        <f>IF(ABS(B8-D8)&lt;0.000001,"OK","≠")</f>
-        <v/>
-      </c>
-      <c r="D8" s="12" t="n">
+      <c r="C8" s="12" t="n">
         <v>0.009861</v>
       </c>
+      <c r="D8" s="4">
+        <f>IF(ABS(B8-C8)&lt;0.000001,"OK","check")</f>
+        <v/>
+      </c>
       <c r="E8" s="10">
-        <f>ACCRUE(DATE(2026,7,15),DATE(2026,7,16),100,"SIMPLE",$B$5,"I")</f>
+        <f>ACCRUE(DATE(2026,7,15),DATE(2026,7,16),100,"SIMPLE",$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ON, weekend (17-Jul)</t>
+          <t>ON, over a weekend</t>
         </is>
       </c>
       <c r="B9" s="11" t="n"/>
-      <c r="C9" s="4">
-        <f>IF(ABS(B9-D9)&lt;0.000001,"OK","≠")</f>
-        <v/>
-      </c>
-      <c r="D9" s="12" t="n">
+      <c r="C9" s="12" t="n">
         <v>0.029583</v>
       </c>
+      <c r="D9" s="4">
+        <f>IF(ABS(B9-C9)&lt;0.000001,"OK","check")</f>
+        <v/>
+      </c>
       <c r="E9" s="10">
-        <f>ACCRUE(DATE(2026,7,17),DATE(2026,7,20),100,"SIMPLE",$B$5,"I")</f>
+        <f>ACCRUE(DATE(2026,7,17),DATE(2026,7,20),100,"SIMPLE",$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ON, holiday bridge (02-Jul)</t>
+          <t>ON, holiday bridge</t>
         </is>
       </c>
       <c r="B10" s="11" t="n"/>
-      <c r="C10" s="4">
-        <f>IF(ABS(B10-D10)&lt;0.000001,"OK","≠")</f>
-        <v/>
-      </c>
-      <c r="D10" s="12" t="n">
+      <c r="C10" s="12" t="n">
         <v>0.039444</v>
       </c>
+      <c r="D10" s="4">
+        <f>IF(ABS(B10-C10)&lt;0.000001,"OK","check")</f>
+        <v/>
+      </c>
       <c r="E10" s="10">
-        <f>ACCRUE(DATE(2026,7,2),DATE(2026,7,6),100,"SIMPLE",$B$5,"I")</f>
+        <f>ACCRUE(DATE(2026,7,2),DATE(2026,7,6),100,"SIMPLE",$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Period simple (Jul-Oct)</t>
+          <t>Period, simple</t>
         </is>
       </c>
       <c r="B11" s="11" t="n"/>
-      <c r="C11" s="4">
-        <f>IF(ABS(B11-D11)&lt;0.000001,"OK","≠")</f>
-        <v/>
-      </c>
-      <c r="D11" s="12" t="n">
+      <c r="C11" s="12" t="n">
         <v>0.85375</v>
       </c>
+      <c r="D11" s="4">
+        <f>IF(ABS(B11-C11)&lt;0.000001,"OK","check")</f>
+        <v/>
+      </c>
       <c r="E11" s="10">
-        <f>ACCRUE(DATE(2026,7,1),DATE(2026,10,1),100,"SIMPLE",$B$5,"I")</f>
+        <f>ACCRUE(DATE(2026,7,1),DATE(2026,10,1),100,"SIMPLE",$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Period compound (Jul-Oct)</t>
+          <t>Period, compounding</t>
         </is>
       </c>
       <c r="B12" s="11" t="n"/>
-      <c r="C12" s="4">
-        <f>IF(ABS(B12-D12)&lt;0.000001,"OK","≠")</f>
-        <v/>
-      </c>
-      <c r="D12" s="12" t="n">
+      <c r="C12" s="12" t="n">
         <v>0.857325</v>
       </c>
+      <c r="D12" s="4">
+        <f>IF(ABS(B12-C12)&lt;0.000001,"OK","check")</f>
+        <v/>
+      </c>
       <c r="E12" s="10">
-        <f>ACCRUE(DATE(2026,7,1),DATE(2026,10,1),100,"COMPOUND",$B$5,"I")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Compound + principal</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="4">
-        <f>IF(ABS(B13-D13)&lt;0.000001,"OK","≠")</f>
-        <v/>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>100.857325</v>
-      </c>
-      <c r="E13" s="10">
-        <f>ACCRUE(DATE(2026,7,1),DATE(2026,10,1),100,"COMPOUND",$B$5,"PI")</f>
-        <v/>
+        <f>ACCRUE(DATE(2026,7,1),DATE(2026,10,1),100,"COMPOUND",$B$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>3 · SWAP — $375mm @3.15%, July, receive-fixed</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>3 · SWAP MONTH ($375mm @3.15%, Jul, RCV) — three legs</t>
-        </is>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>FIXED leg</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="12" t="n">
+        <v>1.017187</v>
+      </c>
+      <c r="D15" s="4">
+        <f>IF(ABS(B15-C15)&lt;0.000001,"OK","check")</f>
+        <v/>
+      </c>
+      <c r="E15" s="10">
+        <f>SWAP(DATE(2026,7,1),DATE(2026,8,1),375,3.15,$B$5,"FIXED")</f>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>FIXED leg</t>
+          <t>FLOAT leg</t>
         </is>
       </c>
       <c r="B16" s="11" t="n"/>
-      <c r="C16" s="4">
-        <f>IF(ABS(B16-D16)&lt;0.000001,"OK","≠")</f>
-        <v/>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>1.017187</v>
+      <c r="C16" s="12" t="n">
+        <v>1.142773</v>
+      </c>
+      <c r="D16" s="4">
+        <f>IF(ABS(B16-C16)&lt;0.000001,"OK","check")</f>
+        <v/>
       </c>
       <c r="E16" s="10">
-        <f>SWAP_NET(DATE(2026,7,1),DATE(2026,8,1),375,3.15,$B$5,"RCV","FIXED")</f>
+        <f>SWAP(DATE(2026,7,1),DATE(2026,8,1),375,3.15,$B$5,"FLOAT")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>FLOAT leg</t>
+          <t>NET (fixed-float)</t>
         </is>
       </c>
       <c r="B17" s="11" t="n"/>
-      <c r="C17" s="4">
-        <f>IF(ABS(B17-D17)&lt;0.000001,"OK","≠")</f>
-        <v/>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>1.142773</v>
+      <c r="C17" s="12" t="n">
+        <v>-0.125585</v>
+      </c>
+      <c r="D17" s="4">
+        <f>IF(ABS(B17-C17)&lt;0.000001,"OK","check")</f>
+        <v/>
       </c>
       <c r="E17" s="10">
-        <f>SWAP_NET(DATE(2026,7,1),DATE(2026,8,1),375,3.15,$B$5,"RCV","FLOAT")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>NET</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="4">
-        <f>IF(ABS(B18-D18)&lt;0.000001,"OK","≠")</f>
-        <v/>
-      </c>
-      <c r="D18" s="12" t="n">
-        <v>-0.125585</v>
-      </c>
-      <c r="E18" s="10">
-        <f>SWAP_NET(DATE(2026,7,1),DATE(2026,8,1),375,3.15,$B$5,"RCV","NET")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>NET = FIXED − FLOAT (RCV).</t>
-        </is>
+        <f>SWAP(DATE(2026,7,1),DATE(2026,8,1),375,3.15,$B$5,"NET")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>